<commit_message>
docs(mvp0): Caso #0 baseline — fila tracker + plantilla captura
Juan como beta #0 en Pipeline; checklist baseline, screening y stack Fase 0.
</commit_message>
<xml_diff>
--- a/estrategia_2026/MVP0_Beta_Tracker.xlsx
+++ b/estrategia_2026/MVP0_Beta_Tracker.xlsx
@@ -93,7 +93,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +115,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -152,7 +157,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -224,6 +229,12 @@
     </xf>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -513,114 +524,122 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Invitaciones enviadas</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
+      <c r="C4" s="14" t="inlineStr"/>
+      <c r="D4" s="14" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Confirmados (sí)</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
+      <c r="C5" s="14" t="inlineStr"/>
+      <c r="D5" s="14" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>Onboarding completado</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
+      <c r="C6" s="14" t="inlineStr"/>
+      <c r="D6" s="14" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>Protocolos entregados</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
+      <c r="C7" s="14" t="inlineStr"/>
+      <c r="D7" s="14" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>Consultas RAG (filas log)</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
+      <c r="C8" s="14" t="inlineStr"/>
+      <c r="D8" s="14" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>% auto + caveat (RAG)</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>≥70%</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
+      <c r="C9" s="14" t="inlineStr"/>
+      <c r="D9" s="14" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>Gaps promovidos</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>Caso #0 iniciado</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>Intención de pago (Feedback)</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
+      <c r="C11" s="14" t="inlineStr"/>
+      <c r="D11" s="14" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Referido espontáneo</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
+      <c r="C12" s="14" t="inlineStr"/>
+      <c r="D12" s="14" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -747,23 +766,75 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="11">
-      <c r="A5" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="18" t="n"/>
-      <c r="C5" s="18" t="n"/>
-      <c r="D5" s="18" t="n"/>
-      <c r="E5" s="18" t="n"/>
-      <c r="F5" s="18" t="n"/>
-      <c r="G5" s="18" t="n"/>
-      <c r="H5" s="18" t="n"/>
-      <c r="I5" s="18" t="n"/>
-      <c r="J5" s="18" t="n"/>
-      <c r="K5" s="18" t="n"/>
-      <c r="L5" s="18" t="n"/>
-      <c r="M5" s="18" t="n"/>
-      <c r="N5" s="18" t="n"/>
-      <c r="O5" s="18" t="n"/>
+      <c r="A5" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="B5" s="27" t="inlineStr">
+        <is>
+          <t>Juan Josué H. (Caso #0)</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="inlineStr">
+        <is>
+          <t>completar</t>
+        </is>
+      </c>
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>completar</t>
+        </is>
+      </c>
+      <c r="E5" s="26" t="inlineStr">
+        <is>
+          <t>Querétaro</t>
+        </is>
+      </c>
+      <c r="F5" s="26" t="inlineStr">
+        <is>
+          <t>Ciática + energía + estética + longevidad</t>
+        </is>
+      </c>
+      <c r="G5" s="26" t="inlineStr">
+        <is>
+          <t>Baseline en curso</t>
+        </is>
+      </c>
+      <c r="H5" s="26" t="inlineStr">
+        <is>
+          <t>SÍ — psiq (litio/quetiapina) + antec. oncológico</t>
+        </is>
+      </c>
+      <c r="I5" s="26" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="J5" s="26" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="K5" s="26" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="L5" s="26" t="inlineStr">
+        <is>
+          <t>Fase 0 (ver Caso0_Baseline.md)</t>
+        </is>
+      </c>
+      <c r="M5" s="26" t="inlineStr"/>
+      <c r="N5" s="26" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="O5" s="26" t="inlineStr">
+        <is>
+          <t>Caso #0 fundador · iniciado 2026-06-07 · MVP0_Caso0_Baseline.md</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="11">
       <c r="A6" s="19" t="n">
@@ -991,7 +1062,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>Una fila por pregunta pasada por concierge_mvp.py / hv-rag-api. decision_id = prod log.</t>
         </is>
@@ -1140,15 +1211,31 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="11">
-      <c r="A5" s="18" t="n"/>
-      <c r="B5" s="18" t="n"/>
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Juan Josué (Caso #0)</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>0 — baseline</t>
+        </is>
+      </c>
       <c r="C5" s="18" t="n"/>
       <c r="D5" s="18" t="n"/>
       <c r="E5" s="18" t="n"/>
       <c r="F5" s="18" t="n"/>
       <c r="G5" s="18" t="n"/>
-      <c r="H5" s="18" t="n"/>
-      <c r="I5" s="18" t="n"/>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="I5" s="18" t="inlineStr">
+        <is>
+          <t>Día 0 — capturar antes de semana 1</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="11">
       <c r="A6" s="19" t="n"/>

</xml_diff>

<commit_message>
docs(mvp0): baseline Caso #0 con labs e imagen lumbar reales
Resume estudios oct-2025 y RM/RX feb-2025; protocolo borrador en repo.
</commit_message>
<xml_diff>
--- a/estrategia_2026/MVP0_Beta_Tracker.xlsx
+++ b/estrategia_2026/MVP0_Beta_Tracker.xlsx
@@ -489,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" style="11" min="1" max="1"/>
@@ -606,16 +606,8 @@
       <c r="B10" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="14" t="inlineStr">
-        <is>
-          <t>Caso #0 iniciado</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="C10" s="14" t="inlineStr"/>
+      <c r="D10" s="14" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
@@ -640,6 +632,28 @@
       </c>
       <c r="C12" s="14" t="inlineStr"/>
       <c r="D12" s="14" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Caso #0</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Iniciado</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -779,10 +793,8 @@
           <t>completar</t>
         </is>
       </c>
-      <c r="D5" s="26" t="inlineStr">
-        <is>
-          <t>completar</t>
-        </is>
+      <c r="D5" s="26" t="n">
+        <v>44</v>
       </c>
       <c r="E5" s="26" t="inlineStr">
         <is>
@@ -806,12 +818,12 @@
       </c>
       <c r="I5" s="26" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="J5" s="26" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Sí — 7-oct-2025</t>
         </is>
       </c>
       <c r="K5" s="26" t="inlineStr">
@@ -832,7 +844,7 @@
       </c>
       <c r="O5" s="26" t="inlineStr">
         <is>
-          <t>Caso #0 fundador · iniciado 2026-06-07 · MVP0_Caso0_Baseline.md</t>
+          <t>Caso #0 · labs+RM/RX feb-oct 2025 · MVP0_Caso0_Baseline.md · foto pendiente</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(mvp0): doctrina, Caso #0 y playbook concierge manual
Añade la operación MVP-0 (triage, entregas, clearance, tracker) y actualiza
playbook, scripts WhatsApp e inventario de producto para la beta manual.
</commit_message>
<xml_diff>
--- a/estrategia_2026/MVP0_Beta_Tracker.xlsx
+++ b/estrategia_2026/MVP0_Beta_Tracker.xlsx
@@ -785,12 +785,12 @@
       </c>
       <c r="B5" s="27" t="inlineStr">
         <is>
-          <t>Juan Josué H. (Caso #0)</t>
+          <t>Juan Josué Hernández Tapia (Caso #0)</t>
         </is>
       </c>
       <c r="C5" s="26" t="inlineStr">
         <is>
-          <t>completar</t>
+          <t>+52 442 202 2540</t>
         </is>
       </c>
       <c r="D5" s="26" t="n">
@@ -808,7 +808,7 @@
       </c>
       <c r="G5" s="26" t="inlineStr">
         <is>
-          <t>Baseline en curso</t>
+          <t>protocolo_entregado</t>
         </is>
       </c>
       <c r="H5" s="26" t="inlineStr">
@@ -823,28 +823,32 @@
       </c>
       <c r="J5" s="26" t="inlineStr">
         <is>
-          <t>Sí — 7-oct-2025</t>
+          <t>Sí — 7-oct-2025 + RM feb-2025</t>
         </is>
       </c>
       <c r="K5" s="26" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>No</t>
         </is>
       </c>
       <c r="L5" s="26" t="inlineStr">
         <is>
-          <t>Fase 0 (ver Caso0_Baseline.md)</t>
-        </is>
-      </c>
-      <c r="M5" s="26" t="inlineStr"/>
+          <t>Wolverine</t>
+        </is>
+      </c>
+      <c r="M5" s="26" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
       <c r="N5" s="26" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Psiquiatra OK 2026-06-07 (suplementos + péptidos inyectables, vista psiq.) · ayuno/litio sin aclarar · médico aliado HV pendiente · C1 desde 2026-06-09</t>
         </is>
       </c>
       <c r="O5" s="26" t="inlineStr">
         <is>
-          <t>Caso #0 · labs+RM/RX feb-oct 2025 · MVP0_Caso0_Baseline.md · foto pendiente</t>
+          <t>C1 sem2: resveratrol OK · sueño 4→5 · energía 3→4 · spermidine 2026-06-23 · señal positiva</t>
         </is>
       </c>
     </row>
@@ -1050,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="11" min="1" max="1"/>
@@ -1134,6 +1138,50 @@
       <c r="K4" s="20" t="inlineStr">
         <is>
           <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Caso #0 / Juan</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>¿puedo hacer ayuno 16:8 si tomo litio?</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>caveat</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr"/>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>4932b68c996b</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr"/>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K5" s="14" t="inlineStr">
+        <is>
+          <t>litio + ayuno — derivar psiquiatra</t>
         </is>
       </c>
     </row>

</xml_diff>